<commit_message>
상태 시트 초안: UnitState.xlsx(PlayerState·EliteState·BossState)
- Boss 탭을 BossState로 바꾸고 Key 열 추가, 4단계(Idle 10000·Rage 7000·Frenzy 4000·Desperate 1000)
- PlayerState(12001~ Stun·Poison·Bleed), EliteState(13001~, 행 없음) 추가
- REGISTRY에 File 열 추가, 세 시트는 UnitState.xlsx 하나로 묶음
- UnitStat Type에 Elite 추가(설명)
- tables/Boss.xlsx·csv/Boss.csv 삭제

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDH3mwZmVtgx1ALhFj2DHN
</commit_message>
<xml_diff>
--- a/tables/REGISTRY.xlsx
+++ b/tables/REGISTRY.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,7 +445,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>한 행 = 시트 하나. Parent·ParentKey는 이 시트 행이 매달리는 상위 시트와 그 열, Uses는 라이브러리처럼 참조하는 시트. Active = N이면 그 시트를 읽지 않는다.</t>
+          <t>한 행 = 시트 하나. Parent·ParentKey는 이 시트 행이 매달리는 상위 시트와 그 열, Uses는 라이브러리처럼 참조하는 시트. File은 저장소 tables/의 xlsx 파일 이름(확장자 제외). 대부분 파일 1개 = 시트 1개이고, PlayerState·EliteState·BossState는 UnitState.xlsx 하나에 시트로 나뉠어 들어감. Active = N이면 그 시트를 읽지 않는다.</t>
         </is>
       </c>
     </row>
@@ -546,6 +546,11 @@
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Active</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>File</t>
         </is>
       </c>
     </row>
@@ -596,6 +601,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>REGISTRY</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -644,6 +654,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -692,6 +707,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -740,6 +760,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>UnitStat</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -788,6 +813,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Attack</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -836,6 +866,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -884,6 +919,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -932,6 +972,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -980,6 +1025,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -987,12 +1037,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>보스 페이즈</t>
+          <t>보스 상태</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Boss</t>
+          <t>BossState</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1026,6 +1076,11 @@
       <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Y</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>UnitState</t>
         </is>
       </c>
     </row>
@@ -1076,6 +1131,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1122,6 +1182,117 @@
       <c r="J18" s="2" t="inlineStr">
         <is>
           <t>Y</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>StageLayer</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>11013</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>플레이어 상태</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>PlayerState</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>UnitStat</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>UnitID</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>12001~</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>UnitState</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>11014</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>엘리트 상태</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>EliteState</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>UnitStat</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>UnitID</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>13001~</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>UnitState</t>
         </is>
       </c>
     </row>

</xml_diff>